<commit_message>
Aura: techo y kit SIPCOR verificados; ajuste de dólar del kit y faltantes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PL4fade9uMUQLM1tmUvUUs
</commit_message>
<xml_diff>
--- a/URBANSIP/AURA/Aura_Precio_Venta.xlsx
+++ b/URBANSIP/AURA/Aura_Precio_Venta.xlsx
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>44896.7</v>
+        <v>45123.8</v>
       </c>
     </row>
     <row r="7">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2550</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="8">
@@ -601,7 +601,6 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Aura Esencial: presupuesto v1 ítem por ítem; corrección de mano de obra
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PL4fade9uMUQLM1tmUvUUs
</commit_message>
<xml_diff>
--- a/URBANSIP/AURA/Aura_Precio_Venta.xlsx
+++ b/URBANSIP/AURA/Aura_Precio_Venta.xlsx
@@ -546,11 +546,11 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>263.83</v>
+        <v>180.29</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Planilla de mano de obra: 263,83. El Excel de costos usa 340 como referencia.</t>
+          <t>Corregido: $20.400.000 de jornales / $1.550 / 73 m². El 263,83 contaba dos veces el montaje del kit.</t>
         </is>
       </c>
     </row>

</xml_diff>